<commit_message>
Release Lizenzfinder V1.19 mit GitHub Pages
</commit_message>
<xml_diff>
--- a/versions/aenderungshistorie/lizenzfinder_versionshistorie.xlsx
+++ b/versions/aenderungshistorie/lizenzfinder_versionshistorie.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Uebersicht" sheetId="1" r:id="R93bba77dcd8c4f78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Versionshistorie" sheetId="2" r:id="R5c1da946f55648e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit-Register" sheetId="3" r:id="R447df182ed6844e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listen" sheetId="4" r:id="R2db69143f8824a61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Uebersicht" sheetId="1" r:id="R60ef92182b1e405c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Versionshistorie" sheetId="2" r:id="R73b0c349cde24898"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit-Register" sheetId="3" r:id="R84c3fc4e8f5a46a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listen" sheetId="4" r:id="R248cc75460e24d9c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -450,7 +450,7 @@
         <x:v>Aktuelle Version</x:v>
       </x:c>
       <x:c r="B4" s="14" t="str">
-        <x:v>1.17.20260819-codex</x:v>
+        <x:v>1.19.20260819-codex</x:v>
       </x:c>
       <x:c r="C4" s="25"/>
       <x:c r="D4" s="27" t="str">
@@ -472,7 +472,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B5" s="14" t="str">
-        <x:v>Release Candidate nach Feinschliff, Netzwerk-Waechter und Doku-Update</x:v>
+        <x:v>Release Candidate nach V1.19-Feinschliff, Browserpruefung und Doku-Update</x:v>
       </x:c>
       <x:c r="C5" s="25"/>
       <x:c r="D5" s="14" t="str">
@@ -480,11 +480,11 @@
       </x:c>
       <x:c r="E5" s="14" t="n">
         <x:f>COUNTA(Versionshistorie!$A$2:$A$200)</x:f>
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="F5" s="14" t="n">
         <x:f>E5</x:f>
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="G5" s="14" t="str">
         <x:v>Anzahl dokumentierter Staende</x:v>
@@ -552,11 +552,11 @@
       </x:c>
       <x:c r="E8" s="14" t="n">
         <x:f>COUNTIF(Versionshistorie!$G$2:$G$200,"Archiviert")</x:f>
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F8" s="14" t="n">
         <x:f>E8</x:f>
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G8" s="14" t="str">
         <x:v>Gesicherte Vorversionen</x:v>
@@ -1232,7 +1232,7 @@
         <x:v>Johannes Koch / Codex</x:v>
       </x:c>
       <x:c r="G18" s="14" t="str">
-        <x:v>Freigabekandidat</x:v>
+        <x:v>Archiviert</x:v>
       </x:c>
       <x:c r="H18" s="14" t="str">
         <x:v>Feinabstand unter Navigation erhoeht; About- und Footer-Texte reduziert; Netzwerk-Waechter und CSP ergaenzt; sichtbare Badges lokal als SVG erzeugt; Schatten im Vermerkbereich entfernt; twillo-Hinweis ruhiger gestaltet.</x:v>
@@ -1244,34 +1244,78 @@
         <x:v>Build-, Release- und Browserpruefung vorgesehen; fachliche Endabnahme, manuelle Tastatur-/Fokuspruefung und GitHub-Push offen</x:v>
       </x:c>
       <x:c r="K18" s="14" t="str">
-        <x:v>GitHub veroeffentlichen, Remote pruefen und fachliche Endabnahme durchfuehren</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="15" hidden="0" customHeight="1">
-      <x:c r="A19" s="14"/>
-      <x:c r="B19" s="15"/>
-      <x:c r="C19" s="14"/>
-      <x:c r="D19" s="14"/>
-      <x:c r="E19" s="14"/>
-      <x:c r="F19" s="14"/>
-      <x:c r="G19" s="14"/>
-      <x:c r="H19" s="14"/>
-      <x:c r="I19" s="14"/>
-      <x:c r="J19" s="14"/>
-      <x:c r="K19" s="14"/>
-    </x:row>
-    <x:row r="20" ht="15" hidden="0" customHeight="1">
-      <x:c r="A20" s="14"/>
-      <x:c r="B20" s="15"/>
-      <x:c r="C20" s="14"/>
-      <x:c r="D20" s="14"/>
-      <x:c r="E20" s="14"/>
-      <x:c r="F20" s="14"/>
-      <x:c r="G20" s="14"/>
-      <x:c r="H20" s="14"/>
-      <x:c r="I20" s="14"/>
-      <x:c r="J20" s="14"/>
-      <x:c r="K20" s="14"/>
+        <x:v>Durch V1.18 abgeloest</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A19" s="14" t="str">
+        <x:v>1.18.20260819-codex</x:v>
+      </x:c>
+      <x:c r="B19" s="15" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="C19" s="14" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D19" s="14" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="E19" s="14" t="str">
+        <x:v>codex</x:v>
+      </x:c>
+      <x:c r="F19" s="14" t="str">
+        <x:v>Johannes Koch / Codex</x:v>
+      </x:c>
+      <x:c r="G19" s="14" t="str">
+        <x:v>Archiviert</x:v>
+      </x:c>
+      <x:c r="H19" s="14" t="str">
+        <x:v>Header-Infofeld entfernt; persistente Speicherung entfernt; Netzwerk-Waechter auf Selbsttest entschärft; URL-Validierung und Clipboard-Fallback ergaenzt; About/Footer und Doppellizenzierung nachgezogen.</x:v>
+      </x:c>
+      <x:c r="I19" s="14" t="str">
+        <x:v>Sicherheit; Datenschutz; Netzwerk; Lizenz; UX; Versionierung</x:v>
+      </x:c>
+      <x:c r="J19" s="14" t="str">
+        <x:v>Build-, Release- und Browserpruefung bestanden; sandboxed iframe, localStorage, URL-Schutz und Copy-Fallback geprueft; fachliche Endabnahme und manuelle Tastatur-/Fokuspruefung offen</x:v>
+      </x:c>
+      <x:c r="K19" s="14" t="str">
+        <x:v>Durch V1.19 abgeloest</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A20" s="14" t="str">
+        <x:v>1.19.20260819-codex</x:v>
+      </x:c>
+      <x:c r="B20" s="15" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="C20" s="14" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D20" s="14" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="E20" s="14" t="str">
+        <x:v>codex</x:v>
+      </x:c>
+      <x:c r="F20" s="14" t="str">
+        <x:v>Johannes Koch / Codex</x:v>
+      </x:c>
+      <x:c r="G20" s="14" t="str">
+        <x:v>Freigabekandidat</x:v>
+      </x:c>
+      <x:c r="H20" s="14" t="str">
+        <x:v>Copyright-Zeichen auf MIT-Lizenztext beschraenkt; About-Panel scrollbar und per Escape schliessbar gemacht; Footer benennt Codex/OpenAI; dynamisches Jahr und verbesserte Quellenwarnung ergaenzt; GitHub-Pages-Einstieg, Workflow, README und Vorlagen vorbereitet.</x:v>
+      </x:c>
+      <x:c r="I20" s="14" t="str">
+        <x:v>Text; Barrierearmut; UX; Lizenz; Datenschutz; GitHub; Versionierung</x:v>
+      </x:c>
+      <x:c r="J20" s="14" t="str">
+        <x:v>Build-, Release- und Browserpruefung bestanden; Copyright-Suche, 500px-Panel, Escape-Fokus, 2027-Jahr, aria-invalid, Pages-index und V1.18-Regressionen geprueft</x:v>
+      </x:c>
+      <x:c r="K20" s="14" t="str">
+        <x:v>Fachliche Endabnahme, manuelle Tastatur-/Fokuspruefung und GitHub-Push nach Freigabe</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="14"/>
@@ -1837,29 +1881,57 @@
         <x:v>mit Auflagen</x:v>
       </x:c>
       <x:c r="F18" s="14" t="str">
-        <x:v>Feinschliff und Netzwerk-Waechter umgesetzt; Build-, Release- und Browserpruefung vorgesehen; GitHub-Push bleibt bis zur Freigabe offen.</x:v>
+        <x:v>Feinschliff und Netzwerk-Waechter umgesetzt; durch V1.18 technisch entschaerft und abgeloest.</x:v>
       </x:c>
       <x:c r="G18" s="14" t="str">
         <x:v>audits/RELEASE_AUDIT_V1_17_20260819.md; Lizenzfinder-App-V1_17_20260819-codex.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="15" hidden="0" customHeight="1">
-      <x:c r="A19" s="14"/>
-      <x:c r="B19" s="15"/>
-      <x:c r="C19" s="14"/>
-      <x:c r="D19" s="14"/>
-      <x:c r="E19" s="14"/>
-      <x:c r="F19" s="14"/>
-      <x:c r="G19" s="14"/>
-    </x:row>
-    <x:row r="20" ht="15" hidden="0" customHeight="1">
-      <x:c r="A20" s="14"/>
-      <x:c r="B20" s="15"/>
-      <x:c r="C20" s="14"/>
-      <x:c r="D20" s="14"/>
-      <x:c r="E20" s="14"/>
-      <x:c r="F20" s="14"/>
-      <x:c r="G20" s="14"/>
+    <x:row r="19" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A19" s="14" t="str">
+        <x:v>A-018</x:v>
+      </x:c>
+      <x:c r="B19" s="15" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="C19" s="14" t="str">
+        <x:v>1.18.20260819-codex</x:v>
+      </x:c>
+      <x:c r="D19" s="14" t="str">
+        <x:v>Release</x:v>
+      </x:c>
+      <x:c r="E19" s="14" t="str">
+        <x:v>mit Auflagen</x:v>
+      </x:c>
+      <x:c r="F19" s="14" t="str">
+        <x:v>V1.18-Haertung umgesetzt; durch V1.19 mit About-Panel- und Textfeinschliff abgeloest.</x:v>
+      </x:c>
+      <x:c r="G19" s="14" t="str">
+        <x:v>audits/RELEASE_AUDIT_V1_18_20260819.md; Lizenzfinder-App-V1_18_20260819-codex.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A20" s="14" t="str">
+        <x:v>A-019</x:v>
+      </x:c>
+      <x:c r="B20" s="15" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="C20" s="14" t="str">
+        <x:v>1.19.20260819-codex</x:v>
+      </x:c>
+      <x:c r="D20" s="14" t="str">
+        <x:v>Release</x:v>
+      </x:c>
+      <x:c r="E20" s="14" t="str">
+        <x:v>mit Auflagen</x:v>
+      </x:c>
+      <x:c r="F20" s="14" t="str">
+        <x:v>V1.19-Feinschliff und GitHub-Pages-Vorbereitung umgesetzt; Build-, Release- und Browserpruefung bestanden; fachliche Endabnahme und manuelle Tastatur-/Fokuspruefung bleiben offen.</x:v>
+      </x:c>
+      <x:c r="G20" s="14" t="str">
+        <x:v>audits/RELEASE_AUDIT_V1_19_20260819.md; Lizenzfinder-App-V1_19_20260819-codex.html</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="14"/>

</xml_diff>

<commit_message>
Release Lizenzfinder V1.20 About-Ergaenzung
</commit_message>
<xml_diff>
--- a/versions/aenderungshistorie/lizenzfinder_versionshistorie.xlsx
+++ b/versions/aenderungshistorie/lizenzfinder_versionshistorie.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Uebersicht" sheetId="1" r:id="R60ef92182b1e405c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Versionshistorie" sheetId="2" r:id="R73b0c349cde24898"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit-Register" sheetId="3" r:id="R84c3fc4e8f5a46a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listen" sheetId="4" r:id="R248cc75460e24d9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Uebersicht" sheetId="1" r:id="R67a6f11867714914"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Versionshistorie" sheetId="2" r:id="R02f0dc18e8d24a3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit-Register" sheetId="3" r:id="R2576228ebfb14f32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listen" sheetId="4" r:id="Rde21e15800bc43e3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -450,7 +450,7 @@
         <x:v>Aktuelle Version</x:v>
       </x:c>
       <x:c r="B4" s="14" t="str">
-        <x:v>1.19.20260819-codex</x:v>
+        <x:v>1.20.20260819-codex</x:v>
       </x:c>
       <x:c r="C4" s="25"/>
       <x:c r="D4" s="27" t="str">
@@ -472,7 +472,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B5" s="14" t="str">
-        <x:v>Release Candidate nach V1.19-Feinschliff, Browserpruefung und Doku-Update</x:v>
+        <x:v>Release Candidate nach V1.20-Link- und Entstehungsergaenzung</x:v>
       </x:c>
       <x:c r="C5" s="25"/>
       <x:c r="D5" s="14" t="str">
@@ -480,11 +480,11 @@
       </x:c>
       <x:c r="E5" s="14" t="n">
         <x:f>COUNTA(Versionshistorie!$A$2:$A$200)</x:f>
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F5" s="14" t="n">
         <x:f>E5</x:f>
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="G5" s="14" t="str">
         <x:v>Anzahl dokumentierter Staende</x:v>
@@ -552,11 +552,11 @@
       </x:c>
       <x:c r="E8" s="14" t="n">
         <x:f>COUNTIF(Versionshistorie!$G$2:$G$200,"Archiviert")</x:f>
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="F8" s="14" t="n">
         <x:f>E8</x:f>
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G8" s="14" t="str">
         <x:v>Gesicherte Vorversionen</x:v>
@@ -1302,7 +1302,7 @@
         <x:v>Johannes Koch / Codex</x:v>
       </x:c>
       <x:c r="G20" s="14" t="str">
-        <x:v>Freigabekandidat</x:v>
+        <x:v>Archiviert</x:v>
       </x:c>
       <x:c r="H20" s="14" t="str">
         <x:v>Copyright-Zeichen auf MIT-Lizenztext beschraenkt; About-Panel scrollbar und per Escape schliessbar gemacht; Footer benennt Codex/OpenAI; dynamisches Jahr und verbesserte Quellenwarnung ergaenzt; GitHub-Pages-Einstieg, Workflow, README und Vorlagen vorbereitet.</x:v>
@@ -1314,21 +1314,43 @@
         <x:v>Build-, Release- und Browserpruefung bestanden; Copyright-Suche, 500px-Panel, Escape-Fokus, 2027-Jahr, aria-invalid, Pages-index und V1.18-Regressionen geprueft</x:v>
       </x:c>
       <x:c r="K20" s="14" t="str">
-        <x:v>Fachliche Endabnahme, manuelle Tastatur-/Fokuspruefung und GitHub-Push nach Freigabe</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="15" hidden="0" customHeight="1">
-      <x:c r="A21" s="14"/>
-      <x:c r="B21" s="15"/>
-      <x:c r="C21" s="14"/>
-      <x:c r="D21" s="14"/>
-      <x:c r="E21" s="14"/>
-      <x:c r="F21" s="14"/>
-      <x:c r="G21" s="14"/>
-      <x:c r="H21" s="14"/>
-      <x:c r="I21" s="14"/>
-      <x:c r="J21" s="14"/>
-      <x:c r="K21" s="14"/>
+        <x:v>Durch V1.20 abgeloest</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="66" hidden="0" customHeight="1">
+      <x:c r="A21" s="14" t="str">
+        <x:v>1.20.20260819-codex</x:v>
+      </x:c>
+      <x:c r="B21" s="15" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="C21" s="14" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D21" s="14" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E21" s="14" t="str">
+        <x:v>codex</x:v>
+      </x:c>
+      <x:c r="F21" s="14" t="str">
+        <x:v>Johannes Koch / Codex</x:v>
+      </x:c>
+      <x:c r="G21" s="14" t="str">
+        <x:v>Freigabekandidat</x:v>
+      </x:c>
+      <x:c r="H21" s="14" t="str">
+        <x:v>MIT License im About-Panel mit der OSI-Lizenzseite verlinkt; Entstehungsabschnitt zu Vibe-Coding, Claude, Codex und redaktioneller Verantwortung ergaenzt; Browsercheck-Pfade aktualisiert.</x:v>
+      </x:c>
+      <x:c r="I21" s="14" t="str">
+        <x:v>Text; Lizenz; Transparenz; GitHub; Versionierung</x:v>
+      </x:c>
+      <x:c r="J21" s="14" t="str">
+        <x:v>Build-, Release- und Browserpruefung bestanden; MIT-Link, Entstehungsabschnitt, Sprachumschaltung und bestehende Kernlogik geprueft</x:v>
+      </x:c>
+      <x:c r="K21" s="14" t="str">
+        <x:v>Fachliche Endabnahme und manuelle Tastatur-/Fokuspruefung nach Freigabe</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="14"/>
@@ -1933,14 +1955,28 @@
         <x:v>audits/RELEASE_AUDIT_V1_19_20260819.md; Lizenzfinder-App-V1_19_20260819-codex.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="15" hidden="0" customHeight="1">
-      <x:c r="A21" s="14"/>
-      <x:c r="B21" s="15"/>
-      <x:c r="C21" s="14"/>
-      <x:c r="D21" s="14"/>
-      <x:c r="E21" s="14"/>
-      <x:c r="F21" s="14"/>
-      <x:c r="G21" s="14"/>
+    <x:row r="21" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A21" s="14" t="str">
+        <x:v>A-020</x:v>
+      </x:c>
+      <x:c r="B21" s="15" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="C21" s="14" t="str">
+        <x:v>1.20.20260819-codex</x:v>
+      </x:c>
+      <x:c r="D21" s="14" t="str">
+        <x:v>Release</x:v>
+      </x:c>
+      <x:c r="E21" s="14" t="str">
+        <x:v>mit Auflagen</x:v>
+      </x:c>
+      <x:c r="F21" s="14" t="str">
+        <x:v>MIT-Link und Entstehungsabschnitt umgesetzt; Build-, Release- und Browserpruefung bestanden; fachliche Endabnahme und manuelle Tastatur-/Fokuspruefung bleiben offen.</x:v>
+      </x:c>
+      <x:c r="G21" s="14" t="str">
+        <x:v>audits/RELEASE_AUDIT_V1_20_20260819.md; Lizenzfinder-App-V1_20_20260819-codex.html</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="14"/>

</xml_diff>

<commit_message>
Release Lizenzfinder V1.21 Footer und About-Dialog
</commit_message>
<xml_diff>
--- a/versions/aenderungshistorie/lizenzfinder_versionshistorie.xlsx
+++ b/versions/aenderungshistorie/lizenzfinder_versionshistorie.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Uebersicht" sheetId="1" r:id="R67a6f11867714914"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Versionshistorie" sheetId="2" r:id="R02f0dc18e8d24a3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit-Register" sheetId="3" r:id="R2576228ebfb14f32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listen" sheetId="4" r:id="Rde21e15800bc43e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Uebersicht" sheetId="1" r:id="R0567667f5d33493d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Versionshistorie" sheetId="2" r:id="R1afe69360aa34849"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit-Register" sheetId="3" r:id="R85f8e4fec87e4e68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listen" sheetId="4" r:id="R3b3918bdc9dd4dd4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -450,7 +450,7 @@
         <x:v>Aktuelle Version</x:v>
       </x:c>
       <x:c r="B4" s="14" t="str">
-        <x:v>1.20.20260819-codex</x:v>
+        <x:v>1.21.20260819-codex</x:v>
       </x:c>
       <x:c r="C4" s="25"/>
       <x:c r="D4" s="27" t="str">
@@ -472,7 +472,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B5" s="14" t="str">
-        <x:v>Release Candidate nach V1.20-Link- und Entstehungsergaenzung</x:v>
+        <x:v>Release Candidate nach V1.21-Footer-Transparenzkorrektur</x:v>
       </x:c>
       <x:c r="C5" s="25"/>
       <x:c r="D5" s="14" t="str">
@@ -480,11 +480,11 @@
       </x:c>
       <x:c r="E5" s="14" t="n">
         <x:f>COUNTA(Versionshistorie!$A$2:$A$200)</x:f>
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="F5" s="14" t="n">
         <x:f>E5</x:f>
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G5" s="14" t="str">
         <x:v>Anzahl dokumentierter Staende</x:v>
@@ -552,11 +552,11 @@
       </x:c>
       <x:c r="E8" s="14" t="n">
         <x:f>COUNTIF(Versionshistorie!$G$2:$G$200,"Archiviert")</x:f>
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F8" s="14" t="n">
         <x:f>E8</x:f>
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G8" s="14" t="str">
         <x:v>Gesicherte Vorversionen</x:v>
@@ -1337,7 +1337,7 @@
         <x:v>Johannes Koch / Codex</x:v>
       </x:c>
       <x:c r="G21" s="14" t="str">
-        <x:v>Freigabekandidat</x:v>
+        <x:v>Archiviert</x:v>
       </x:c>
       <x:c r="H21" s="14" t="str">
         <x:v>MIT License im About-Panel mit der OSI-Lizenzseite verlinkt; Entstehungsabschnitt zu Vibe-Coding, Claude, Codex und redaktioneller Verantwortung ergaenzt; Browsercheck-Pfade aktualisiert.</x:v>
@@ -1349,21 +1349,43 @@
         <x:v>Build-, Release- und Browserpruefung bestanden; MIT-Link, Entstehungsabschnitt, Sprachumschaltung und bestehende Kernlogik geprueft</x:v>
       </x:c>
       <x:c r="K21" s="14" t="str">
+        <x:v>Durch V1.21 abgeloest</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="66" hidden="0" customHeight="1">
+      <x:c r="A22" s="14" t="str">
+        <x:v>1.21.20260819-codex</x:v>
+      </x:c>
+      <x:c r="B22" s="15" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="C22" s="14" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D22" s="14" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="E22" s="14" t="str">
+        <x:v>codex</x:v>
+      </x:c>
+      <x:c r="F22" s="14" t="str">
+        <x:v>Johannes Koch / Codex</x:v>
+      </x:c>
+      <x:c r="G22" s="14" t="str">
+        <x:v>Freigabekandidat</x:v>
+      </x:c>
+      <x:c r="H22" s="14" t="str">
+        <x:v>Footer- und Transparenztexte nennen Claude/Anthropic und Codex/OpenAI; App-Name bleibt Lizenzfinder; About-Bereich an BITTE-STIL-Struktur angeglichen und Button in die Fusszeile verschoben.</x:v>
+      </x:c>
+      <x:c r="I22" s="14" t="str">
+        <x:v>Text; Lizenz; Transparenz; GitHub; Versionierung</x:v>
+      </x:c>
+      <x:c r="J22" s="14" t="str">
+        <x:v>Build-, Release- und Browserpruefung bestanden; Footer-Text, About-Dialog, englische Ansicht und bestehende Kernlogik geprueft</x:v>
+      </x:c>
+      <x:c r="K22" s="14" t="str">
         <x:v>Fachliche Endabnahme und manuelle Tastatur-/Fokuspruefung nach Freigabe</x:v>
       </x:c>
-    </x:row>
-    <x:row r="22" ht="15" hidden="0" customHeight="1">
-      <x:c r="A22" s="14"/>
-      <x:c r="B22" s="15"/>
-      <x:c r="C22" s="14"/>
-      <x:c r="D22" s="14"/>
-      <x:c r="E22" s="14"/>
-      <x:c r="F22" s="14"/>
-      <x:c r="G22" s="14"/>
-      <x:c r="H22" s="14"/>
-      <x:c r="I22" s="14"/>
-      <x:c r="J22" s="14"/>
-      <x:c r="K22" s="14"/>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="14"/>
@@ -1978,14 +2000,28 @@
         <x:v>audits/RELEASE_AUDIT_V1_20_20260819.md; Lizenzfinder-App-V1_20_20260819-codex.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="15" hidden="0" customHeight="1">
-      <x:c r="A22" s="14"/>
-      <x:c r="B22" s="15"/>
-      <x:c r="C22" s="14"/>
-      <x:c r="D22" s="14"/>
-      <x:c r="E22" s="14"/>
-      <x:c r="F22" s="14"/>
-      <x:c r="G22" s="14"/>
+    <x:row r="22" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A22" s="14" t="str">
+        <x:v>A-021</x:v>
+      </x:c>
+      <x:c r="B22" s="15" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="C22" s="14" t="str">
+        <x:v>1.21.20260819-codex</x:v>
+      </x:c>
+      <x:c r="D22" s="14" t="str">
+        <x:v>Release</x:v>
+      </x:c>
+      <x:c r="E22" s="14" t="str">
+        <x:v>mit Auflagen</x:v>
+      </x:c>
+      <x:c r="F22" s="14" t="str">
+        <x:v>Footer- und Transparenztexte auf Claude/Anthropic und Codex/OpenAI erweitert; About-Dialog an BITTE-STIL-Struktur angeglichen; App-Name Lizenzfinder beibehalten; Build-, Release- und Browserpruefung bestanden.</x:v>
+      </x:c>
+      <x:c r="G22" s="14" t="str">
+        <x:v>audits/RELEASE_AUDIT_V1_21_20260819.md; Lizenzfinder-App-V1_21_20260819-codex.html</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="14"/>

</xml_diff>

<commit_message>
Release Lizenzfinder V1.22 Dialogskalierung
</commit_message>
<xml_diff>
--- a/versions/aenderungshistorie/lizenzfinder_versionshistorie.xlsx
+++ b/versions/aenderungshistorie/lizenzfinder_versionshistorie.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Uebersicht" sheetId="1" r:id="R0567667f5d33493d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Versionshistorie" sheetId="2" r:id="R1afe69360aa34849"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit-Register" sheetId="3" r:id="R85f8e4fec87e4e68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listen" sheetId="4" r:id="R3b3918bdc9dd4dd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Uebersicht" sheetId="1" r:id="R608858e650f04759"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Versionshistorie" sheetId="2" r:id="Rc3f8a3efb79747f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit-Register" sheetId="3" r:id="R4d8435ca8ec34267"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listen" sheetId="4" r:id="R2a02519d6f7946b4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -450,7 +450,7 @@
         <x:v>Aktuelle Version</x:v>
       </x:c>
       <x:c r="B4" s="14" t="str">
-        <x:v>1.21.20260819-codex</x:v>
+        <x:v>1.22.20260819-codex</x:v>
       </x:c>
       <x:c r="C4" s="25"/>
       <x:c r="D4" s="27" t="str">
@@ -467,12 +467,12 @@
       </x:c>
       <x:c r="H4" s="27" t="str"/>
     </x:row>
-    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="26" t="str">
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B5" s="14" t="str">
-        <x:v>Release Candidate nach V1.21-Footer-Transparenzkorrektur</x:v>
+        <x:v>Release Candidate nach V1.22-Dialogskalierung</x:v>
       </x:c>
       <x:c r="C5" s="25"/>
       <x:c r="D5" s="14" t="str">
@@ -480,11 +480,11 @@
       </x:c>
       <x:c r="E5" s="14" t="n">
         <x:f>COUNTA(Versionshistorie!$A$2:$A$200)</x:f>
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F5" s="14" t="n">
         <x:f>E5</x:f>
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="G5" s="14" t="str">
         <x:v>Anzahl dokumentierter Staende</x:v>
@@ -552,11 +552,11 @@
       </x:c>
       <x:c r="E8" s="14" t="n">
         <x:f>COUNTIF(Versionshistorie!$G$2:$G$200,"Archiviert")</x:f>
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="F8" s="14" t="n">
         <x:f>E8</x:f>
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G8" s="14" t="str">
         <x:v>Gesicherte Vorversionen</x:v>
@@ -1372,7 +1372,7 @@
         <x:v>Johannes Koch / Codex</x:v>
       </x:c>
       <x:c r="G22" s="14" t="str">
-        <x:v>Freigabekandidat</x:v>
+        <x:v>Archiviert</x:v>
       </x:c>
       <x:c r="H22" s="14" t="str">
         <x:v>Footer- und Transparenztexte nennen Claude/Anthropic und Codex/OpenAI; App-Name bleibt Lizenzfinder; About-Bereich an BITTE-STIL-Struktur angeglichen und Button in die Fusszeile verschoben.</x:v>
@@ -1384,21 +1384,43 @@
         <x:v>Build-, Release- und Browserpruefung bestanden; Footer-Text, About-Dialog, englische Ansicht und bestehende Kernlogik geprueft</x:v>
       </x:c>
       <x:c r="K22" s="14" t="str">
+        <x:v>Durch V1.22 abgeloest</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="66" hidden="0" customHeight="1">
+      <x:c r="A23" s="14" t="str">
+        <x:v>1.22.20260819-codex</x:v>
+      </x:c>
+      <x:c r="B23" s="15" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="C23" s="14" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D23" s="14" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E23" s="14" t="str">
+        <x:v>codex</x:v>
+      </x:c>
+      <x:c r="F23" s="14" t="str">
+        <x:v>Johannes Koch / Codex</x:v>
+      </x:c>
+      <x:c r="G23" s="14" t="str">
+        <x:v>Freigabekandidat</x:v>
+      </x:c>
+      <x:c r="H23" s="14" t="str">
+        <x:v>Dialog 'Ueber diese Anwendung' kleiner skaliert und visuell enger an den BITTE-STIL-Baukasten angeglichen; Footer-Button-Struktur bleibt erhalten.</x:v>
+      </x:c>
+      <x:c r="I23" s="14" t="str">
+        <x:v>UX; Gestaltung; Versionierung</x:v>
+      </x:c>
+      <x:c r="J23" s="14" t="str">
+        <x:v>Build-, Release- und Browserpruefung bestanden; About-Dialog, Sprachumschaltung und bestehende Kernlogik geprueft</x:v>
+      </x:c>
+      <x:c r="K23" s="14" t="str">
         <x:v>Fachliche Endabnahme und manuelle Tastatur-/Fokuspruefung nach Freigabe</x:v>
       </x:c>
-    </x:row>
-    <x:row r="23" ht="15" hidden="0" customHeight="1">
-      <x:c r="A23" s="14"/>
-      <x:c r="B23" s="15"/>
-      <x:c r="C23" s="14"/>
-      <x:c r="D23" s="14"/>
-      <x:c r="E23" s="14"/>
-      <x:c r="F23" s="14"/>
-      <x:c r="G23" s="14"/>
-      <x:c r="H23" s="14"/>
-      <x:c r="I23" s="14"/>
-      <x:c r="J23" s="14"/>
-      <x:c r="K23" s="14"/>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="14"/>
@@ -2023,14 +2045,28 @@
         <x:v>audits/RELEASE_AUDIT_V1_21_20260819.md; Lizenzfinder-App-V1_21_20260819-codex.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="15" hidden="0" customHeight="1">
-      <x:c r="A23" s="14"/>
-      <x:c r="B23" s="15"/>
-      <x:c r="C23" s="14"/>
-      <x:c r="D23" s="14"/>
-      <x:c r="E23" s="14"/>
-      <x:c r="F23" s="14"/>
-      <x:c r="G23" s="14"/>
+    <x:row r="23" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A23" s="14" t="str">
+        <x:v>A-022</x:v>
+      </x:c>
+      <x:c r="B23" s="15" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="C23" s="14" t="str">
+        <x:v>1.22.20260819-codex</x:v>
+      </x:c>
+      <x:c r="D23" s="14" t="str">
+        <x:v>Release</x:v>
+      </x:c>
+      <x:c r="E23" s="14" t="str">
+        <x:v>mit Auflagen</x:v>
+      </x:c>
+      <x:c r="F23" s="14" t="str">
+        <x:v>About-Dialog auf BITTE-STIL-naehere Groesse reduziert; Build-, Release- und Browserpruefung bestanden; fachliche Endabnahme und manuelle Tastatur-/Fokuspruefung bleiben offen.</x:v>
+      </x:c>
+      <x:c r="G23" s="14" t="str">
+        <x:v>audits/RELEASE_AUDIT_V1_22_20260819.md; Lizenzfinder-App-V1_22_20260819-codex.html</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="14"/>

</xml_diff>